<commit_message>
Clarifie la JDV utilisée pour ageMin/ageMax de ror-healthcareservice-patient-type
- Fixe extension:ageRange.value[x].low/high.system sur http://unitsofmeasure.org
  et lie low/high.code en required binding vers JDV_J37-UcumUniteTemps
  (qui pointe désormais vers UCUM depuis le 29/09/2024), au lieu de l'ancien
  système TRE_R247-UcumUniteMesure.
- Ajout de l'alias $JDV-J37-UcumUniteTemps dans aliases.fsh.
- Mise à jour de l'exemple RORHealthcareServiceExemple (système UCUM au lieu
  de TRE_R247) et de RORQuestionnaireOffreMCO (answerValueSet sur JDV_J37,
  system UCUM sur les initial valueCoding, correction d'un guillemet
  parasite sur les codes #d/#a).
- Mise à jour de la documentation (search_param.md, specifications_techniques_3.md)
  pour référencer JDV_J37-UcumUniteTemps/UCUM et corriger le schéma
  https -> http sur unitsofmeasure.org.

Fixes #445

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> e3a7c2b4eb458504f986319d79c918b13fedeea1
</commit_message>
<xml_diff>
--- a/update-dependencies-fr-core-annuaire/ig/StructureDefinition-ror-healthcareservice-patient-type.xlsx
+++ b/update-dependencies-fr-core-annuaire/ig/StructureDefinition-ror-healthcareservice-patient-type.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1194" uniqueCount="218">
   <si>
     <t>Property</t>
   </si>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-23T08:09:55+00:00</t>
+    <t>2026-08-20T16:34:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -463,6 +463,162 @@
     <t>./low</t>
   </si>
   <si>
+    <t>Extension.extension:ageRange.value[x].low.id</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].low.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].low.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].low.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].low.value</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].low.value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">decimal
+</t>
+  </si>
+  <si>
+    <t>Numerical value (with implicit precision)</t>
+  </si>
+  <si>
+    <t>The value of the measured amount. The value includes an implicit precision in the presentation of the value.</t>
+  </si>
+  <si>
+    <t>The implicit precision in the value should always be honored. Monetary values have their own rules for handling precision (refer to standard accounting text books).</t>
+  </si>
+  <si>
+    <t>Precision is handled implicitly in almost all cases of measurement.</t>
+  </si>
+  <si>
+    <t>Quantity.value</t>
+  </si>
+  <si>
+    <t>PQ.value, CO.value, MO.value, IVL.high or IVL.low depending on the value</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].low.comparator</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].low.comparator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">code
+</t>
+  </si>
+  <si>
+    <t>&lt; | &lt;= | &gt;= | &gt; - how to understand the value</t>
+  </si>
+  <si>
+    <t>Not allowed to be used in this context</t>
+  </si>
+  <si>
+    <t>Note that FHIR strings SHALL NOT exceed 1MB in size</t>
+  </si>
+  <si>
+    <t>Need a framework for handling measures where the value is &lt;5ug/L or &gt;400mg/L due to the limitations of measuring methodology.</t>
+  </si>
+  <si>
+    <t>If there is no comparator, then there is no modification of the value</t>
+  </si>
+  <si>
+    <t>How the Quantity should be understood and represented.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/quantity-comparator|4.0.1</t>
+  </si>
+  <si>
+    <t>Quantity.comparator</t>
+  </si>
+  <si>
+    <t>IVL properties</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].low.unit</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].low.unit</t>
+  </si>
+  <si>
+    <t>Unit representation</t>
+  </si>
+  <si>
+    <t>A human-readable form of the unit.</t>
+  </si>
+  <si>
+    <t>There are many representations for units of measure and in many contexts, particular representations are fixed and required. I.e. mcg for micrograms.</t>
+  </si>
+  <si>
+    <t>Quantity.unit</t>
+  </si>
+  <si>
+    <t>PQ.unit</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].low.system</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].low.system</t>
+  </si>
+  <si>
+    <t>System that defines coded unit form</t>
+  </si>
+  <si>
+    <t>The identification of the system that provides the coded form of the unit.</t>
+  </si>
+  <si>
+    <t>see http://en.wikipedia.org/wiki/Uniform_resource_identifier</t>
+  </si>
+  <si>
+    <t>Need to know the system that defines the coded form of the unit.</t>
+  </si>
+  <si>
+    <t>http://unitsofmeasure.org</t>
+  </si>
+  <si>
+    <t>Quantity.system</t>
+  </si>
+  <si>
+    <t>ele-1
+qty-3</t>
+  </si>
+  <si>
+    <t>CO.codeSystem, PQ.translation.codeSystem</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].low.code</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].low.code</t>
+  </si>
+  <si>
+    <t>Coded form of the unit</t>
+  </si>
+  <si>
+    <t>A computer processable form of the unit in some unit representation system.</t>
+  </si>
+  <si>
+    <t>The preferred system is UCUM, but SNOMED CT can also be used (for customary units) or ISO 4217 for currency.  The context of use may additionally require a code from a particular system.</t>
+  </si>
+  <si>
+    <t>Need a computable form of the unit that is fixed across all forms. UCUM provides this for quantities, but SNOMED CT provides many units of interest.</t>
+  </si>
+  <si>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J37-UcumUniteTemps/FHIR/JDV-J37-UcumUniteTemps</t>
+  </si>
+  <si>
+    <t>Quantity.code</t>
+  </si>
+  <si>
+    <t>PQ.code, MO.currency, PQ.translation.code</t>
+  </si>
+  <si>
     <t>Extension.extension:ageRange.value[x].high</t>
   </si>
   <si>
@@ -482,6 +638,48 @@
   </si>
   <si>
     <t>./high</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].high.id</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].high.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].high.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].high.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].high.value</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].high.value</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].high.comparator</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].high.comparator</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].high.unit</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].high.unit</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].high.system</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].high.system</t>
+  </si>
+  <si>
+    <t>Extension.extension:ageRange.value[x].high.code</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x].high.code</t>
   </si>
   <si>
     <t>base64Binary
@@ -793,11 +991,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL20"/>
+  <dimension ref="A1:AL34"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="42.0390625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="31.94140625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="45.80078125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="37.328125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="17.4140625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="10.83984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -810,7 +1008,7 @@
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="13.4296875" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="120.28125" customWidth="true" bestFit="true"/>
     <col min="16" max="16" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
@@ -820,19 +1018,19 @@
     <col min="22" max="22" width="15.13671875" customWidth="true" bestFit="true"/>
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="46.3671875" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="82.18359375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="15.59375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="17.33984375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
     <col min="37" max="37" width="74.1328125" customWidth="true" bestFit="true"/>
-    <col min="38" max="38" width="21.4140625" customWidth="true" bestFit="true"/>
+    <col min="38" max="38" width="59.11328125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2670,7 +2868,7 @@
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G18" t="s" s="2">
         <v>84</v>
@@ -2682,20 +2880,18 @@
         <v>76</v>
       </c>
       <c r="J18" t="s" s="2">
-        <v>137</v>
+        <v>76</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>138</v>
+        <v>85</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>147</v>
+        <v>86</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>148</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>149</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
         <v>76</v>
@@ -2744,7 +2940,7 @@
         <v>76</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>150</v>
+        <v>88</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>77</v>
@@ -2753,35 +2949,35 @@
         <v>84</v>
       </c>
       <c r="AI18" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AJ18" t="s" s="2">
-        <v>143</v>
+        <v>76</v>
       </c>
       <c r="AK18" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>151</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>109</v>
+        <v>147</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>76</v>
+        <v>131</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G19" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="H19" t="s" s="2">
         <v>76</v>
@@ -2793,16 +2989,16 @@
         <v>76</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>106</v>
+        <v>132</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -2810,7 +3006,7 @@
       </c>
       <c r="Q19" s="2"/>
       <c r="R19" t="s" s="2">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="S19" t="s" s="2">
         <v>76</v>
@@ -2840,31 +3036,31 @@
         <v>76</v>
       </c>
       <c r="AB19" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AC19" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AD19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE19" t="s" s="2">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="AG19" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AH19" t="s" s="2">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="AI19" t="s" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AK19" t="s" s="2">
         <v>76</v>
@@ -2875,10 +3071,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>118</v>
+        <v>149</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>118</v>
+        <v>150</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -2889,7 +3085,7 @@
         <v>77</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H20" t="s" s="2">
         <v>76</v>
@@ -2898,19 +3094,23 @@
         <v>76</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>76</v>
+        <v>137</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L20" t="s" s="2">
         <v>152</v>
       </c>
-      <c r="L20" t="s" s="2">
-        <v>114</v>
-      </c>
       <c r="M20" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
+        <v>153</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="O20" t="s" s="2">
+        <v>155</v>
+      </c>
       <c r="P20" t="s" s="2">
         <v>76</v>
       </c>
@@ -2958,7 +3158,7 @@
         <v>76</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>118</v>
+        <v>156</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>77</v>
@@ -2976,6 +3176,1532 @@
         <v>76</v>
       </c>
       <c r="AL20" t="s" s="2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="B21" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E21" s="2"/>
+      <c r="F21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I21" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="J21" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K21" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="L21" t="s" s="2">
+        <v>161</v>
+      </c>
+      <c r="M21" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="N21" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="O21" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="P21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q21" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="R21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X21" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="Y21" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="Z21" t="s" s="2">
+        <v>167</v>
+      </c>
+      <c r="AA21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF21" t="s" s="2">
+        <v>168</v>
+      </c>
+      <c r="AG21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH21" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ21" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL21" t="s" s="2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="2">
+        <v>170</v>
+      </c>
+      <c r="B22" t="s" s="2">
+        <v>171</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="F22" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G22" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J22" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K22" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="L22" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="M22" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="N22" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="O22" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="P22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q22" s="2"/>
+      <c r="R22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF22" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="AG22" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH22" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI22" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ22" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL22" t="s" s="2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="B23" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="G23" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J23" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K23" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="L23" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="M23" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="O23" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="P23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q23" s="2"/>
+      <c r="R23" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="S23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF23" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="AG23" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH23" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI23" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="AJ23" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL23" t="s" s="2">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="2">
+        <v>187</v>
+      </c>
+      <c r="B24" t="s" s="2">
+        <v>188</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="G24" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J24" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K24" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="L24" t="s" s="2">
+        <v>189</v>
+      </c>
+      <c r="M24" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="N24" t="s" s="2">
+        <v>191</v>
+      </c>
+      <c r="O24" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="P24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q24" s="2"/>
+      <c r="R24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X24" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="Y24" s="2"/>
+      <c r="Z24" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="AA24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF24" t="s" s="2">
+        <v>194</v>
+      </c>
+      <c r="AG24" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH24" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI24" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ24" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL24" t="s" s="2">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="B25" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="G25" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J25" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K25" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="L25" t="s" s="2">
+        <v>198</v>
+      </c>
+      <c r="M25" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="O25" s="2"/>
+      <c r="P25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q25" s="2"/>
+      <c r="R25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF25" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="AG25" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH25" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ25" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="AK25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL25" t="s" s="2">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="2">
+        <v>203</v>
+      </c>
+      <c r="B26" t="s" s="2">
+        <v>204</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G26" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K26" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="L26" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="M26" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="N26" s="2"/>
+      <c r="O26" s="2"/>
+      <c r="P26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q26" s="2"/>
+      <c r="R26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF26" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="AG26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH26" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL26" t="s" s="2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="2">
+        <v>205</v>
+      </c>
+      <c r="B27" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K27" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="L27" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="M27" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="O27" s="2"/>
+      <c r="P27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q27" s="2"/>
+      <c r="R27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB27" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AF27" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AG27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ27" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK27" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL27" t="s" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="2">
+        <v>207</v>
+      </c>
+      <c r="B28" t="s" s="2">
+        <v>208</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E28" s="2"/>
+      <c r="F28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G28" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J28" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K28" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="L28" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="M28" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="N28" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="O28" t="s" s="2">
+        <v>155</v>
+      </c>
+      <c r="P28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q28" s="2"/>
+      <c r="R28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF28" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="AG28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH28" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ28" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL28" t="s" s="2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s" s="2">
+        <v>209</v>
+      </c>
+      <c r="B29" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E29" s="2"/>
+      <c r="F29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I29" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="J29" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K29" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="L29" t="s" s="2">
+        <v>161</v>
+      </c>
+      <c r="M29" t="s" s="2">
+        <v>162</v>
+      </c>
+      <c r="N29" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="O29" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="P29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q29" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="R29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X29" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="Y29" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="Z29" t="s" s="2">
+        <v>167</v>
+      </c>
+      <c r="AA29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF29" t="s" s="2">
+        <v>168</v>
+      </c>
+      <c r="AG29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH29" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI29" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ29" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL29" t="s" s="2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s" s="2">
+        <v>211</v>
+      </c>
+      <c r="B30" t="s" s="2">
+        <v>212</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E30" s="2"/>
+      <c r="F30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G30" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J30" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K30" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="L30" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="M30" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>163</v>
+      </c>
+      <c r="O30" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="P30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q30" s="2"/>
+      <c r="R30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF30" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="AG30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH30" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI30" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ30" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK30" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL30" t="s" s="2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s" s="2">
+        <v>213</v>
+      </c>
+      <c r="B31" t="s" s="2">
+        <v>214</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E31" s="2"/>
+      <c r="F31" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="G31" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J31" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K31" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="L31" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="M31" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="N31" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="O31" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="P31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q31" s="2"/>
+      <c r="R31" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="S31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF31" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="AG31" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH31" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI31" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="AJ31" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK31" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL31" t="s" s="2">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="B32" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E32" s="2"/>
+      <c r="F32" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="G32" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J32" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="K32" t="s" s="2">
+        <v>160</v>
+      </c>
+      <c r="L32" t="s" s="2">
+        <v>189</v>
+      </c>
+      <c r="M32" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="N32" t="s" s="2">
+        <v>191</v>
+      </c>
+      <c r="O32" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="P32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q32" s="2"/>
+      <c r="R32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X32" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="Y32" s="2"/>
+      <c r="Z32" t="s" s="2">
+        <v>193</v>
+      </c>
+      <c r="AA32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF32" t="s" s="2">
+        <v>194</v>
+      </c>
+      <c r="AG32" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH32" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI32" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ32" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK32" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL32" t="s" s="2">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="B33" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E33" s="2"/>
+      <c r="F33" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="G33" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K33" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="L33" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="M33" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="N33" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="O33" s="2"/>
+      <c r="P33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q33" s="2"/>
+      <c r="R33" t="s" s="2">
+        <v>3</v>
+      </c>
+      <c r="S33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF33" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AG33" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH33" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK33" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL33" t="s" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="B34" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E34" s="2"/>
+      <c r="F34" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G34" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K34" t="s" s="2">
+        <v>217</v>
+      </c>
+      <c r="L34" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="M34" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="N34" s="2"/>
+      <c r="O34" s="2"/>
+      <c r="P34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q34" s="2"/>
+      <c r="R34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF34" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="AG34" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH34" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI34" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ34" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AK34" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AL34" t="s" s="2">
         <v>110</v>
       </c>
     </row>

</xml_diff>